<commit_message>
Update master handwritten study notes, 5-stage study roadmap, and add new Excel workbooks (Conditional Formatting, Financial, Store)
</commit_message>
<xml_diff>
--- a/Excel Formulas - Copy.xlsx
+++ b/Excel Formulas - Copy.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20375"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucky\Desktop\Advance Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96E99E44-BAD0-4589-9C54-7D8D644E7DA6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DF3BC04-88BC-471F-B4BF-2AAB430BCF50}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" tabRatio="913" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -54,7 +54,7 @@
     <definedName name="Transction_Type" localSheetId="7">COUNTIFS!$B$2:$B$13</definedName>
     <definedName name="Transction_Type">SUMIFS!$B$2:$B$13</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterate="1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1234,78 +1234,6 @@
   </cellStyles>
   <dxfs count="17">
     <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="13" formatCode="0%"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -1444,6 +1372,29 @@
       </fill>
     </dxf>
     <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="13" formatCode="0%"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -1459,6 +1410,55 @@
         </bottom>
         <vertical/>
         <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -1846,16 +1846,16 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{12DBE826-1808-4D80-9CB0-1499606D48A4}" name="Table2" displayName="Table2" ref="A1:F13" totalsRowShown="0" headerRowDxfId="16" headerRowBorderDxfId="15" tableBorderDxfId="14">
   <autoFilter ref="A1:F13" xr:uid="{5913976F-9E3A-4049-BBC2-D51A9CC64B71}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B4606057-A0FF-43BB-87D7-A62A74071A24}" name="Date" dataDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{48180429-BFC1-4668-93F8-9FF29D0A4CFA}" name="EMP" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{BD99BBC6-46ED-4623-8381-CC6D196A6490}" name="BASIC SALARY" dataDxfId="13"/>
-    <tableColumn id="4" xr3:uid="{93D96351-5684-49CB-9791-0C02F46644C0}" name="BONUS" dataDxfId="4" dataCellStyle="Percent">
+    <tableColumn id="1" xr3:uid="{B4606057-A0FF-43BB-87D7-A62A74071A24}" name="Date" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{48180429-BFC1-4668-93F8-9FF29D0A4CFA}" name="EMP" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{BD99BBC6-46ED-4623-8381-CC6D196A6490}" name="BASIC SALARY" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{93D96351-5684-49CB-9791-0C02F46644C0}" name="BONUS" dataDxfId="10" dataCellStyle="Percent">
       <calculatedColumnFormula>IF(C2&gt;=20000,"Yes","No")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{C9161BDA-97C8-437B-BD1E-6C45FEAC7BC0}" name="BONUS2" dataDxfId="3">
+    <tableColumn id="5" xr3:uid="{C9161BDA-97C8-437B-BD1E-6C45FEAC7BC0}" name="BONUS2" dataDxfId="9">
       <calculatedColumnFormula>IF(C2&gt;=20000,"10%","5%")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{54B4A8D7-ADC0-4BB5-AD33-6560A5A940F9}" name="BONUS3" dataDxfId="2">
+    <tableColumn id="6" xr3:uid="{54B4A8D7-ADC0-4BB5-AD33-6560A5A940F9}" name="BONUS3" dataDxfId="8">
       <calculatedColumnFormula>IF(Table2[[#This Row],[BASIC SALARY]]&gt;=20000,"1000","500")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1864,12 +1864,12 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="sk" displayName="sk" ref="A1:C16" totalsRowShown="0" headerRowDxfId="10" headerRowBorderDxfId="9" tableBorderDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="sk" displayName="sk" ref="A1:C16" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3">
   <autoFilter ref="A1:C16" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Employee Code" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Designation" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Salary" dataDxfId="5" dataCellStyle="Percent"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Employee Code" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Designation" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Salary" dataDxfId="0" dataCellStyle="Percent"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3872,14 +3872,14 @@
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="41">
         <f ca="1">TODAY()</f>
-        <v>46233</v>
+        <v>46241</v>
       </c>
       <c r="B3">
         <v>7</v>
       </c>
       <c r="C3" s="41">
         <f ca="1">A3+B3</f>
-        <v>46240</v>
+        <v>46248</v>
       </c>
       <c r="D3" t="s">
         <v>221</v>
@@ -3888,20 +3888,20 @@
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="41">
         <f ca="1">TODAY()</f>
-        <v>46233</v>
+        <v>46241</v>
       </c>
       <c r="B4">
         <v>5</v>
       </c>
       <c r="C4" s="41">
         <f ca="1">A4-B4</f>
-        <v>46228</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="50">
         <f ca="1">NOW()</f>
-        <v>46233.597055324077</v>
+        <v>46241.623535995372</v>
       </c>
       <c r="C6" t="s">
         <v>222</v>
@@ -3919,7 +3919,7 @@
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9">
         <f ca="1">MONTH(A6)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C9" t="s">
         <v>224</v>
@@ -3928,7 +3928,7 @@
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10">
         <f ca="1">DAY(A6)</f>
-        <v>30</v>
+        <v>7</v>
       </c>
       <c r="C10" t="s">
         <v>225</v>
@@ -3937,7 +3937,7 @@
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="41">
         <f ca="1">DATE(A8,A9,A10)</f>
-        <v>46233</v>
+        <v>46241</v>
       </c>
       <c r="C12" t="s">
         <v>226</v>
@@ -3949,11 +3949,11 @@
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="str">
         <f ca="1">TEXT(A6,"dddd")</f>
-        <v>Thursday</v>
+        <v>Friday</v>
       </c>
       <c r="B14" t="str">
         <f ca="1">TEXT(A6,"mmmm")</f>
-        <v>July</v>
+        <v>August</v>
       </c>
       <c r="C14" t="s">
         <v>227</v>
@@ -3962,39 +3962,39 @@
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="str">
         <f ca="1">TEXT(A12,"ddd")</f>
-        <v>Thu</v>
+        <v>Fri</v>
       </c>
       <c r="B15" t="str">
         <f ca="1">TEXT(A6,"mmm")</f>
-        <v>Jul</v>
+        <v>Aug</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="str">
         <f ca="1">TEXT(A12,"dd")</f>
-        <v>30</v>
+        <v>07</v>
       </c>
       <c r="B16" t="str">
         <f ca="1">TEXT(A6,"mm")</f>
-        <v>07</v>
+        <v>08</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B17" t="str">
         <f ca="1">TEXT(A6,"m")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="str">
         <f ca="1">TEXT(A12,"mmm-yy")</f>
-        <v>Jul-26</v>
+        <v>Aug-26</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20">
         <f ca="1">WEEKDAY(A12,11)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -5312,10 +5312,10 @@
     <mergeCell ref="C2:U2"/>
   </mergeCells>
   <conditionalFormatting sqref="C3:U15">
-    <cfRule type="cellIs" dxfId="12" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="1" operator="equal">
       <formula>"M"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="11" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="2" operator="equal">
       <formula>"F"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6192,11 +6192,11 @@
       </c>
       <c r="F24" s="38">
         <f t="shared" ref="D24:G35" ca="1" si="0">RANDBETWEEN(5000,50000)</f>
-        <v>22081</v>
+        <v>17276</v>
       </c>
       <c r="G24" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>27822</v>
+        <v>27365</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -6214,11 +6214,11 @@
       </c>
       <c r="F25" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>29069</v>
+        <v>49531</v>
       </c>
       <c r="G25" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>7566</v>
+        <v>44842</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -6231,11 +6231,11 @@
       </c>
       <c r="F26" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>48477</v>
+        <v>24286</v>
       </c>
       <c r="G26" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>9690</v>
+        <v>29817</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -6248,11 +6248,11 @@
       </c>
       <c r="F27" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>28359</v>
+        <v>26037</v>
       </c>
       <c r="G27" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>23965</v>
+        <v>18243</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -6263,11 +6263,11 @@
       </c>
       <c r="F28" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>42552</v>
+        <v>34784</v>
       </c>
       <c r="G28" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>20996</v>
+        <v>6313</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -6275,41 +6275,41 @@
       <c r="C29" s="35"/>
       <c r="F29" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>39322</v>
+        <v>39951</v>
       </c>
       <c r="G29" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>21345</v>
+        <v>28737</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="33"/>
       <c r="C30" s="38">
         <f ca="1">RANDBETWEEN(5000,50000)</f>
-        <v>34294</v>
+        <v>30823</v>
       </c>
       <c r="D30" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>42281</v>
+        <v>31958</v>
       </c>
       <c r="E30" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>41664</v>
+        <v>26989</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="21" x14ac:dyDescent="0.35">
       <c r="A31" s="33"/>
       <c r="C31" s="38">
         <f t="shared" ref="C31:C35" ca="1" si="1">RANDBETWEEN(5000,50000)</f>
-        <v>19017</v>
+        <v>31618</v>
       </c>
       <c r="D31" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>14878</v>
+        <v>44336</v>
       </c>
       <c r="E31" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>46108</v>
+        <v>42305</v>
       </c>
       <c r="G31" s="39" t="s">
         <v>151</v>
@@ -6319,60 +6319,60 @@
       <c r="A32" s="33"/>
       <c r="C32" s="38">
         <f t="shared" ca="1" si="1"/>
-        <v>26659</v>
+        <v>39763</v>
       </c>
       <c r="D32" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>48609</v>
+        <v>25786</v>
       </c>
       <c r="E32" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>25484</v>
+        <v>10693</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="33"/>
       <c r="C33" s="38">
         <f t="shared" ca="1" si="1"/>
-        <v>44688</v>
+        <v>42076</v>
       </c>
       <c r="D33" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>16461</v>
+        <v>27604</v>
       </c>
       <c r="E33" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>45748</v>
+        <v>24597</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="34"/>
       <c r="C34" s="38">
         <f t="shared" ca="1" si="1"/>
-        <v>28383</v>
+        <v>16843</v>
       </c>
       <c r="D34" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>25746</v>
+        <v>44499</v>
       </c>
       <c r="E34" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>22511</v>
+        <v>44196</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="34"/>
       <c r="C35" s="38">
         <f t="shared" ca="1" si="1"/>
-        <v>31985</v>
+        <v>9609</v>
       </c>
       <c r="D35" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>32092</v>
+        <v>41779</v>
       </c>
       <c r="E35" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>5074</v>
+        <v>15323</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Organize all solved Excel workbooks into Solved_Files directory
</commit_message>
<xml_diff>
--- a/Excel Formulas - Copy.xlsx
+++ b/Excel Formulas - Copy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucky\Desktop\Advance Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B39966B4-1938-4339-92D0-C2117C0841A3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{094A6523-49CB-41FF-867B-BE82641F47D0}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" tabRatio="913" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" tabRatio="913" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IF FORMULA" sheetId="15" r:id="rId1"/>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="797" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="858" uniqueCount="315">
   <si>
     <t>Ashok Singh</t>
   </si>
@@ -839,6 +839,189 @@
   </si>
   <si>
     <t>Sort</t>
+  </si>
+  <si>
+    <t>ABC</t>
+  </si>
+  <si>
+    <t>HTG</t>
+  </si>
+  <si>
+    <t>RSF</t>
+  </si>
+  <si>
+    <t>IUW</t>
+  </si>
+  <si>
+    <t>GFD</t>
+  </si>
+  <si>
+    <t>HPK</t>
+  </si>
+  <si>
+    <t>TDG</t>
+  </si>
+  <si>
+    <t>OHI</t>
+  </si>
+  <si>
+    <t>MOI</t>
+  </si>
+  <si>
+    <t>HGF</t>
+  </si>
+  <si>
+    <t>IKJ</t>
+  </si>
+  <si>
+    <t>AVS</t>
+  </si>
+  <si>
+    <t>ERR</t>
+  </si>
+  <si>
+    <t>UJH</t>
+  </si>
+  <si>
+    <t>OKJ</t>
+  </si>
+  <si>
+    <t>PLK</t>
+  </si>
+  <si>
+    <t>SDG</t>
+  </si>
+  <si>
+    <t>george</t>
+  </si>
+  <si>
+    <t>herbert</t>
+  </si>
+  <si>
+    <t>hussein</t>
+  </si>
+  <si>
+    <t>walker</t>
+  </si>
+  <si>
+    <t>jefferson</t>
+  </si>
+  <si>
+    <t>wilson</t>
+  </si>
+  <si>
+    <t>earl</t>
+  </si>
+  <si>
+    <t>rudolph</t>
+  </si>
+  <si>
+    <t>milhous</t>
+  </si>
+  <si>
+    <t>baines</t>
+  </si>
+  <si>
+    <t>fitzgerald</t>
+  </si>
+  <si>
+    <t>david</t>
+  </si>
+  <si>
+    <t>s</t>
+  </si>
+  <si>
+    <t>delano</t>
+  </si>
+  <si>
+    <t>clark</t>
+  </si>
+  <si>
+    <t>coolidge</t>
+  </si>
+  <si>
+    <t>gamaliel</t>
+  </si>
+  <si>
+    <t>howard</t>
+  </si>
+  <si>
+    <t>roosevelt</t>
+  </si>
+  <si>
+    <t>mckinley</t>
+  </si>
+  <si>
+    <t>harrison</t>
+  </si>
+  <si>
+    <t>cleveland</t>
+  </si>
+  <si>
+    <t>alan</t>
+  </si>
+  <si>
+    <t>abram</t>
+  </si>
+  <si>
+    <t>birchard</t>
+  </si>
+  <si>
+    <t>simpson</t>
+  </si>
+  <si>
+    <t>johnson</t>
+  </si>
+  <si>
+    <t>lincoln</t>
+  </si>
+  <si>
+    <t>buchanan</t>
+  </si>
+  <si>
+    <t>pierce</t>
+  </si>
+  <si>
+    <t>fillmore</t>
+  </si>
+  <si>
+    <t>taylor</t>
+  </si>
+  <si>
+    <t>knox</t>
+  </si>
+  <si>
+    <t>tyler</t>
+  </si>
+  <si>
+    <t>henry</t>
+  </si>
+  <si>
+    <t>van</t>
+  </si>
+  <si>
+    <t>jackson</t>
+  </si>
+  <si>
+    <t>quincy</t>
+  </si>
+  <si>
+    <t>monroe</t>
+  </si>
+  <si>
+    <t>madison</t>
+  </si>
+  <si>
+    <t>adams</t>
+  </si>
+  <si>
+    <t>washington</t>
+  </si>
+  <si>
+    <t>raj hussein</t>
+  </si>
+  <si>
+    <t>raj</t>
   </si>
 </sst>
 </file>
@@ -1149,7 +1332,7 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1248,6 +1431,7 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1257,6 +1441,26 @@
     <cellStyle name="Percent" xfId="4" builtinId="5"/>
   </cellStyles>
   <dxfs count="17">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -1374,26 +1578,6 @@
         <top/>
         <bottom/>
       </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -1686,8 +1870,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="1813891" y="688939"/>
-          <a:ext cx="5419442" cy="1811711"/>
+          <a:off x="1793838" y="721024"/>
+          <a:ext cx="5254009" cy="1871869"/>
           <a:chOff x="1794184" y="723444"/>
           <a:chExt cx="5151498" cy="1911283"/>
         </a:xfrm>
@@ -1888,12 +2072,12 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="sk" displayName="sk" ref="A1:C16" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="sk" displayName="sk" ref="A1:C16" totalsRowShown="0" headerRowDxfId="7" headerRowBorderDxfId="6" tableBorderDxfId="5">
   <autoFilter ref="A1:C16" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Employee Code" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Designation" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Salary" dataDxfId="0" dataCellStyle="Percent"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Employee Code" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Designation" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Salary" dataDxfId="2" dataCellStyle="Percent"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3890,7 +4074,7 @@
   <dimension ref="A1:G44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="4" width="15.28515625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3916,268 +4100,505 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>152</v>
+        <v>313</v>
+      </c>
+      <c r="B2" t="s">
+        <v>314</v>
+      </c>
+      <c r="C2" t="s">
+        <v>273</v>
       </c>
       <c r="E2" t="s">
         <v>118</v>
+      </c>
+      <c r="F2" t="s">
+        <v>254</v>
+      </c>
+      <c r="G2">
+        <v>986</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>153</v>
       </c>
+      <c r="B3" t="s">
+        <v>271</v>
+      </c>
+      <c r="C3" t="s">
+        <v>274</v>
+      </c>
       <c r="E3" t="s">
         <v>119</v>
+      </c>
+      <c r="F3" t="s">
+        <v>255</v>
+      </c>
+      <c r="G3">
+        <v>987</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>154</v>
       </c>
+      <c r="C4" t="s">
+        <v>275</v>
+      </c>
       <c r="E4" t="s">
         <v>120</v>
+      </c>
+      <c r="F4" t="s">
+        <v>263</v>
+      </c>
+      <c r="G4">
+        <v>985</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>155</v>
       </c>
+      <c r="C5" t="s">
+        <v>272</v>
+      </c>
       <c r="E5" t="s">
         <v>121</v>
+      </c>
+      <c r="F5" t="s">
+        <v>264</v>
+      </c>
+      <c r="G5">
+        <v>748</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>156</v>
       </c>
+      <c r="C6" t="s">
+        <v>276</v>
+      </c>
       <c r="E6" t="s">
         <v>122</v>
+      </c>
+      <c r="F6" t="s">
+        <v>256</v>
+      </c>
+      <c r="G6">
+        <v>854</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>157</v>
       </c>
+      <c r="C7" t="s">
+        <v>277</v>
+      </c>
       <c r="E7" t="s">
         <v>123</v>
+      </c>
+      <c r="F7" t="s">
+        <v>257</v>
+      </c>
+      <c r="G7">
+        <v>965</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>158</v>
       </c>
+      <c r="C8" t="s">
+        <v>278</v>
+      </c>
       <c r="E8" t="s">
         <v>124</v>
+      </c>
+      <c r="F8" t="s">
+        <v>265</v>
+      </c>
+      <c r="G8">
+        <v>655</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>159</v>
       </c>
+      <c r="C9" t="s">
+        <v>279</v>
+      </c>
       <c r="E9" t="s">
         <v>125</v>
+      </c>
+      <c r="F9" t="s">
+        <v>266</v>
+      </c>
+      <c r="G9">
+        <v>321</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>160</v>
       </c>
+      <c r="C10" t="s">
+        <v>280</v>
+      </c>
       <c r="E10" t="s">
         <v>126</v>
+      </c>
+      <c r="F10" t="s">
+        <v>258</v>
+      </c>
+      <c r="G10">
+        <v>955</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>161</v>
       </c>
+      <c r="C11" t="s">
+        <v>281</v>
+      </c>
       <c r="E11" t="s">
         <v>127</v>
+      </c>
+      <c r="F11" t="s">
+        <v>267</v>
+      </c>
+      <c r="G11">
+        <v>965</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>162</v>
       </c>
+      <c r="C12" t="s">
+        <v>282</v>
+      </c>
       <c r="E12" t="s">
         <v>128</v>
+      </c>
+      <c r="F12" t="s">
+        <v>259</v>
+      </c>
+      <c r="G12">
+        <v>965</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>163</v>
       </c>
+      <c r="C13" t="s">
+        <v>283</v>
+      </c>
       <c r="E13" t="s">
         <v>129</v>
+      </c>
+      <c r="F13" t="s">
+        <v>268</v>
+      </c>
+      <c r="G13">
+        <v>857</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>164</v>
       </c>
+      <c r="C14" t="s">
+        <v>284</v>
+      </c>
       <c r="E14" t="s">
         <v>130</v>
+      </c>
+      <c r="F14" t="s">
+        <v>269</v>
+      </c>
+      <c r="G14">
+        <v>965</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>165</v>
       </c>
+      <c r="C15" t="s">
+        <v>285</v>
+      </c>
       <c r="E15" t="s">
         <v>131</v>
+      </c>
+      <c r="F15" t="s">
+        <v>270</v>
+      </c>
+      <c r="G15">
+        <v>147</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>166</v>
       </c>
+      <c r="C16" t="s">
+        <v>286</v>
+      </c>
       <c r="E16" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F16" t="s">
+        <v>260</v>
+      </c>
+      <c r="G16">
+        <v>854</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>167</v>
       </c>
+      <c r="C17" t="s">
+        <v>287</v>
+      </c>
       <c r="E17" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F17" t="s">
+        <v>261</v>
+      </c>
+      <c r="G17">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>168</v>
       </c>
+      <c r="C18" t="s">
+        <v>276</v>
+      </c>
       <c r="E18" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F18" t="s">
+        <v>262</v>
+      </c>
+      <c r="G18">
+        <v>974</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C19" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C20" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C21" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C22" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C23" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C24" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C25" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C26" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C27" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C28" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C29" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C30" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C31" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="C32" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="C33" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="C34" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="C35" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="C36" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="C37" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="C38" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="C39" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="C40" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="C41" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="C42" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="C43" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>194</v>
+      </c>
+      <c r="C44" t="s">
+        <v>312</v>
       </c>
     </row>
   </sheetData>
@@ -4303,13 +4724,19 @@
       <c r="F2" s="1">
         <v>1</v>
       </c>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="K2" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="L2" s="1"/>
+      <c r="G2" s="7">
+        <f>IPMT($C$3/12,F2,$C$5,-$C$4)</f>
+        <v>833.33333333333337</v>
+      </c>
+      <c r="H2" s="7">
+        <f>PPMT($C$3/12,F2,$C$5,-$C$4)</f>
+        <v>9630.704765605522</v>
+      </c>
+      <c r="I2" s="7">
+        <f>PMT($C$3/12,$C$5,-$C$4)</f>
+        <v>10464.038098938856</v>
+      </c>
+      <c r="K2" s="1"/>
       <c r="N2" s="1"/>
       <c r="O2" s="1"/>
     </row>
@@ -4332,9 +4759,18 @@
       <c r="F3" s="1">
         <v>2</v>
       </c>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
+      <c r="G3" s="7">
+        <f t="shared" ref="G3:G11" si="0">IPMT($C$3/12,F3,$C$5,-$C$4)</f>
+        <v>753.07746028662052</v>
+      </c>
+      <c r="H3" s="7">
+        <f t="shared" ref="H3:H11" si="1">PPMT($C$3/12,F3,$C$5,-$C$4)</f>
+        <v>9710.9606386522355</v>
+      </c>
+      <c r="I3" s="7">
+        <f t="shared" ref="I3:I11" si="2">PMT($C$3/12,$C$5,-$C$4)</f>
+        <v>10464.038098938856</v>
+      </c>
       <c r="K3" s="1" t="s">
         <v>91</v>
       </c>
@@ -4364,9 +4800,18 @@
       <c r="F4" s="1">
         <v>3</v>
       </c>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
+      <c r="G4" s="7">
+        <f t="shared" si="0"/>
+        <v>672.15278829785188</v>
+      </c>
+      <c r="H4" s="7">
+        <f t="shared" si="1"/>
+        <v>9791.8853106410024</v>
+      </c>
+      <c r="I4" s="7">
+        <f t="shared" si="2"/>
+        <v>10464.038098938856</v>
+      </c>
       <c r="K4" s="1" t="s">
         <v>83</v>
       </c>
@@ -4396,9 +4841,18 @@
       <c r="F5" s="1">
         <v>4</v>
       </c>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
+      <c r="G5" s="7">
+        <f t="shared" si="0"/>
+        <v>590.55374404251017</v>
+      </c>
+      <c r="H5" s="7">
+        <f t="shared" si="1"/>
+        <v>9873.4843548963454</v>
+      </c>
+      <c r="I5" s="7">
+        <f t="shared" si="2"/>
+        <v>10464.038098938856</v>
+      </c>
       <c r="K5" s="1" t="s">
         <v>85</v>
       </c>
@@ -4417,9 +4871,18 @@
       <c r="F6" s="1">
         <v>5</v>
       </c>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
+      <c r="G6" s="7">
+        <f t="shared" si="0"/>
+        <v>508.2747077517073</v>
+      </c>
+      <c r="H6" s="7">
+        <f t="shared" si="1"/>
+        <v>9955.763391187149</v>
+      </c>
+      <c r="I6" s="7">
+        <f t="shared" si="2"/>
+        <v>10464.038098938856</v>
+      </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
@@ -4428,21 +4891,39 @@
       <c r="B7" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="C7" s="16"/>
+      <c r="C7" s="16">
+        <f>SUM(I2:I11)</f>
+        <v>104640.38098938855</v>
+      </c>
       <c r="F7" s="1">
         <v>6</v>
       </c>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="7"/>
+      <c r="G7" s="7">
+        <f t="shared" si="0"/>
+        <v>425.31001282514779</v>
+      </c>
+      <c r="H7" s="7">
+        <f t="shared" si="1"/>
+        <v>10038.728086113708</v>
+      </c>
+      <c r="I7" s="7">
+        <f t="shared" si="2"/>
+        <v>10464.038098938856</v>
+      </c>
       <c r="K7" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="L7" s="9"/>
+      <c r="L7" s="66">
+        <f>PV(L3/12,L5,-L4)</f>
+        <v>941307.38047503715</v>
+      </c>
       <c r="N7" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O7" s="9"/>
+      <c r="O7" s="9">
+        <f>FV(O3,O5,-O4)</f>
+        <v>78056.16258846609</v>
+      </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
@@ -4456,9 +4937,18 @@
       <c r="F8" s="1">
         <v>7</v>
       </c>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="7"/>
+      <c r="G8" s="7">
+        <f t="shared" si="0"/>
+        <v>341.65394544086683</v>
+      </c>
+      <c r="H8" s="7">
+        <f t="shared" si="1"/>
+        <v>10122.384153497989</v>
+      </c>
+      <c r="I8" s="7">
+        <f t="shared" si="2"/>
+        <v>10464.038098938856</v>
+      </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
@@ -4467,39 +4957,75 @@
       <c r="B9" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="C9" s="7"/>
+      <c r="C9" s="7">
+        <f>SUM(G2:G11)</f>
+        <v>4640.3809893885682</v>
+      </c>
       <c r="E9" s="8"/>
       <c r="F9" s="1">
         <v>8</v>
       </c>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
+      <c r="G9" s="7">
+        <f t="shared" si="0"/>
+        <v>257.30074416171698</v>
+      </c>
+      <c r="H9" s="7">
+        <f t="shared" si="1"/>
+        <v>10206.73735477714</v>
+      </c>
+      <c r="I9" s="7">
+        <f t="shared" si="2"/>
+        <v>10464.038098938856</v>
+      </c>
+      <c r="N9" s="43"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F10" s="1">
         <v>9</v>
       </c>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="7"/>
+      <c r="G10" s="7">
+        <f t="shared" si="0"/>
+        <v>172.24459953857416</v>
+      </c>
+      <c r="H10" s="7">
+        <f t="shared" si="1"/>
+        <v>10291.793499400283</v>
+      </c>
+      <c r="I10" s="7">
+        <f t="shared" si="2"/>
+        <v>10464.038098938856</v>
+      </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C11" s="6"/>
       <c r="F11" s="1">
         <v>10</v>
       </c>
-      <c r="G11" s="7"/>
-      <c r="H11" s="7"/>
-      <c r="I11" s="7"/>
+      <c r="G11" s="7">
+        <f t="shared" si="0"/>
+        <v>86.47965371023848</v>
+      </c>
+      <c r="H11" s="7">
+        <f t="shared" si="1"/>
+        <v>10377.558445228618</v>
+      </c>
+      <c r="I11" s="7">
+        <f t="shared" si="2"/>
+        <v>10464.038098938856</v>
+      </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F12" s="1"/>
       <c r="G12" s="7"/>
       <c r="H12" s="7"/>
       <c r="I12" s="7"/>
+      <c r="N12" s="43"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="G14" s="6">
+        <f>SUM(G11,H11)</f>
+        <v>10464.038098938858</v>
+      </c>
       <c r="H14" s="17"/>
     </row>
     <row r="18" spans="4:4" x14ac:dyDescent="0.25">
@@ -4573,7 +5099,7 @@
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="50">
         <f ca="1">NOW()</f>
-        <v>46245.642577662038</v>
+        <v>46245.66510972222</v>
       </c>
       <c r="C6" t="s">
         <v>222</v>
@@ -5984,10 +6510,10 @@
     <mergeCell ref="C2:U2"/>
   </mergeCells>
   <conditionalFormatting sqref="C3:U15">
-    <cfRule type="cellIs" dxfId="7" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"M"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
       <formula>"F"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6864,11 +7390,11 @@
       </c>
       <c r="F24" s="38">
         <f t="shared" ref="D24:G35" ca="1" si="0">RANDBETWEEN(5000,50000)</f>
-        <v>46027</v>
+        <v>21653</v>
       </c>
       <c r="G24" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>39814</v>
+        <v>44875</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -6886,11 +7412,11 @@
       </c>
       <c r="F25" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>46917</v>
+        <v>6782</v>
       </c>
       <c r="G25" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>33104</v>
+        <v>14479</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -6903,11 +7429,11 @@
       </c>
       <c r="F26" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>13817</v>
+        <v>15175</v>
       </c>
       <c r="G26" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>37023</v>
+        <v>41250</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -6920,11 +7446,11 @@
       </c>
       <c r="F27" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>46572</v>
+        <v>38768</v>
       </c>
       <c r="G27" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>38811</v>
+        <v>41339</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -6935,11 +7461,11 @@
       </c>
       <c r="F28" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>36548</v>
+        <v>44882</v>
       </c>
       <c r="G28" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>36080</v>
+        <v>38092</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -6947,41 +7473,41 @@
       <c r="C29" s="35"/>
       <c r="F29" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>10629</v>
+        <v>16767</v>
       </c>
       <c r="G29" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>6099</v>
+        <v>15458</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="33"/>
       <c r="C30" s="38">
         <f ca="1">RANDBETWEEN(5000,50000)</f>
-        <v>30564</v>
+        <v>6818</v>
       </c>
       <c r="D30" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>12860</v>
+        <v>23515</v>
       </c>
       <c r="E30" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>48916</v>
+        <v>31894</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="21" x14ac:dyDescent="0.35">
       <c r="A31" s="33"/>
       <c r="C31" s="38">
         <f t="shared" ref="C31:C35" ca="1" si="1">RANDBETWEEN(5000,50000)</f>
-        <v>11776</v>
+        <v>46621</v>
       </c>
       <c r="D31" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>33820</v>
+        <v>27355</v>
       </c>
       <c r="E31" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>12024</v>
+        <v>13726</v>
       </c>
       <c r="G31" s="39" t="s">
         <v>151</v>
@@ -6991,60 +7517,60 @@
       <c r="A32" s="33"/>
       <c r="C32" s="38">
         <f t="shared" ca="1" si="1"/>
-        <v>48291</v>
+        <v>15172</v>
       </c>
       <c r="D32" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>13903</v>
+        <v>36211</v>
       </c>
       <c r="E32" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>19583</v>
+        <v>15091</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="33"/>
       <c r="C33" s="38">
         <f t="shared" ca="1" si="1"/>
-        <v>33391</v>
+        <v>18948</v>
       </c>
       <c r="D33" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>48502</v>
+        <v>20592</v>
       </c>
       <c r="E33" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>43925</v>
+        <v>34042</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="34"/>
       <c r="C34" s="38">
         <f t="shared" ca="1" si="1"/>
-        <v>46176</v>
+        <v>6013</v>
       </c>
       <c r="D34" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>34927</v>
+        <v>26014</v>
       </c>
       <c r="E34" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>5077</v>
+        <v>5031</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="34"/>
       <c r="C35" s="38">
         <f t="shared" ca="1" si="1"/>
-        <v>21875</v>
+        <v>35036</v>
       </c>
       <c r="D35" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>19982</v>
+        <v>15526</v>
       </c>
       <c r="E35" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>11710</v>
+        <v>31851</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>